<commit_message>
Update 27 sep. 2026 v1, uden oms. og + 1
</commit_message>
<xml_diff>
--- a/filer_1/10117224_maxi_zoo_denmark_a_s.xlsx
+++ b/filer_1/10117224_maxi_zoo_denmark_a_s.xlsx
@@ -6122,20 +6122,20 @@
         </is>
       </c>
       <c r="B9" s="27">
-        <f>SUM(B5:B8)</f>
+        <f>IF(COUNT('res_raw_10117224'!$F$2,'res_raw_10117224'!$F$3,'res_raw_10117224'!$F$4,'res_raw_10117224'!$F$5)=0,'res_raw_10117224'!$F$6,SUM(B5:B8))</f>
         <v/>
       </c>
       <c r="C9" s="27">
-        <f>SUM(C5:C8)</f>
+        <f>IF(COUNT('res_raw_10117224'!$E$2,'res_raw_10117224'!$E$3,'res_raw_10117224'!$E$4,'res_raw_10117224'!$E$5)=0,'res_raw_10117224'!$E$6,SUM(C5:C8))</f>
         <v/>
       </c>
       <c r="D9" s="27">
-        <f>SUM(D5:D8)</f>
+        <f>IF(COUNT('res_raw_10117224'!$D$2,'res_raw_10117224'!$D$3,'res_raw_10117224'!$D$4,'res_raw_10117224'!$D$5)=0,'res_raw_10117224'!$D$6,SUM(D5:D8))</f>
         <v/>
       </c>
       <c r="F9" s="28" t="inlineStr">
         <is>
-          <t>Beregnet: Nettoomsætning + Andre driftsindt. − Vareforbrug − Andre ext. omk.</t>
+          <t>Beregnet: Nettoomsætning + Andre driftsindt. − Vareforbrug − Andre ext. omk. Er komponenterne ikke indberettet, vises rapporteret bruttoresultat (fsa:GrossResult) direkte.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update 29 sep. 2026 v1
</commit_message>
<xml_diff>
--- a/filer_1/10117224_maxi_zoo_denmark_a_s.xlsx
+++ b/filer_1/10117224_maxi_zoo_denmark_a_s.xlsx
@@ -6122,15 +6122,15 @@
         </is>
       </c>
       <c r="B9" s="27">
-        <f>IF(COUNT('res_raw_10117224'!$F$2,'res_raw_10117224'!$F$3,'res_raw_10117224'!$F$4,'res_raw_10117224'!$F$5)=0,'res_raw_10117224'!$F$6,SUM(B5:B8))</f>
+        <f>IF(ABS((SUM(B5:B8))-'res_raw_10117224'!$F$6)&lt;=2,SUM(B5:B8),'res_raw_10117224'!$F$6)</f>
         <v/>
       </c>
       <c r="C9" s="27">
-        <f>IF(COUNT('res_raw_10117224'!$E$2,'res_raw_10117224'!$E$3,'res_raw_10117224'!$E$4,'res_raw_10117224'!$E$5)=0,'res_raw_10117224'!$E$6,SUM(C5:C8))</f>
+        <f>IF(ABS((SUM(C5:C8))-'res_raw_10117224'!$E$6)&lt;=2,SUM(C5:C8),'res_raw_10117224'!$E$6)</f>
         <v/>
       </c>
       <c r="D9" s="27">
-        <f>IF(COUNT('res_raw_10117224'!$D$2,'res_raw_10117224'!$D$3,'res_raw_10117224'!$D$4,'res_raw_10117224'!$D$5)=0,'res_raw_10117224'!$D$6,SUM(D5:D8))</f>
+        <f>IF(ABS((SUM(D5:D8))-'res_raw_10117224'!$D$6)&lt;=2,SUM(D5:D8),'res_raw_10117224'!$D$6)</f>
         <v/>
       </c>
       <c r="F9" s="28" t="inlineStr">
@@ -6218,15 +6218,15 @@
         </is>
       </c>
       <c r="B13" s="27">
-        <f>SUM(B9:B12)</f>
+        <f>IF(ABS((SUM(B9:B12))-'res_raw_10117224'!$F$11)&lt;=2,SUM(B9:B12),'res_raw_10117224'!$F$11)</f>
         <v/>
       </c>
       <c r="C13" s="27">
-        <f>SUM(C9:C12)</f>
+        <f>IF(ABS((SUM(C9:C12))-'res_raw_10117224'!$E$11)&lt;=2,SUM(C9:C12),'res_raw_10117224'!$E$11)</f>
         <v/>
       </c>
       <c r="D13" s="27">
-        <f>SUM(D9:D12)</f>
+        <f>IF(ABS((SUM(D9:D12))-'res_raw_10117224'!$D$11)&lt;=2,SUM(D9:D12),'res_raw_10117224'!$D$11)</f>
         <v/>
       </c>
       <c r="F13" s="28" t="inlineStr">
@@ -6290,15 +6290,15 @@
         </is>
       </c>
       <c r="B16" s="27">
-        <f>SUM(B13:B15)</f>
+        <f>IF(ABS((SUM(B13:B15))-'res_raw_10117224'!$F$16)&lt;=2,SUM(B13:B15),'res_raw_10117224'!$F$16)</f>
         <v/>
       </c>
       <c r="C16" s="27">
-        <f>SUM(C13:C15)</f>
+        <f>IF(ABS((SUM(C13:C15))-'res_raw_10117224'!$E$16)&lt;=2,SUM(C13:C15),'res_raw_10117224'!$E$16)</f>
         <v/>
       </c>
       <c r="D16" s="27">
-        <f>SUM(D13:D15)</f>
+        <f>IF(ABS((SUM(D13:D15))-'res_raw_10117224'!$D$16)&lt;=2,SUM(D13:D15),'res_raw_10117224'!$D$16)</f>
         <v/>
       </c>
       <c r="F16" s="28" t="inlineStr">

</xml_diff>